<commit_message>
feat(danh bạ): bỏ phạm vi bắt buộc cho QA
</commit_message>
<xml_diff>
--- a/public/templates/phan-quyen-vmp.xlsx
+++ b/public/templates/phan-quyen-vmp.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>STT</t>
   </si>
@@ -56,13 +56,16 @@
     <t>Mã nhân viên hiện không bắt buộc; có thể để trống và bổ sung sau. Hệ thống tạm khớp bằng Họ và tên có dấu, không phân biệt hoa thường và khoảng trắng.</t>
   </si>
   <si>
-    <t>Bốn cột phạm vi nhập mã danh mục chuẩn, nhiều giá trị cách nhau bằng dấu chấm phẩy. Mỗi xưởng phải thuộc một bộ phận đã chọn, mỗi khu vực thuộc một xưởng đã chọn và mỗi line thuộc một khu vực đã chọn.</t>
+    <t>Nhân sự QA để trống bốn cột phạm vi; quyền QA phát sinh từ phân công từng hạng mục.</t>
   </si>
   <si>
-    <t>Muốn cấp toàn bộ ở một tầng, nhập mã lựa chọn Toàn bộ đã được cấu hình trong danh mục; ô trống không có nghĩa là toàn bộ.</t>
+    <t>Các phân loại ngoài QA vẫn phải nhập đủ bộ phận, xưởng, khu vực và line.</t>
   </si>
   <si>
-    <t>Email nhận tài khoản: nếu trùng email của tài khoản hệ thống, danh bạ tự nối đúng user_id. Không dùng chung một email cho hai người.</t>
+    <t>Với phân loại ngoài QA, bốn cột phạm vi nhập mã danh mục chuẩn, nhiều giá trị cách nhau bằng dấu chấm phẩy. Mỗi xưởng phải thuộc một bộ phận đã chọn, mỗi khu vực thuộc một xưởng đã chọn và mỗi line thuộc một khu vực đã chọn.</t>
+  </si>
+  <si>
+    <t>Email chỉ dùng nhận diện ứng viên; Admin phải nối tài khoản trên web trước khi quyền có hiệu lực.</t>
   </si>
   <si>
     <t>Xác nhận gửi email: chọn Có sau khi đã gửi thông tin tài khoản; không có chức năng tự động gửi email trong file này.</t>
@@ -8118,7 +8121,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -8204,6 +8207,11 @@
         <v>26</v>
       </c>
     </row>
+    <row r="17" ht="30" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>